<commit_message>
7.1.1 workbook update Tony
</commit_message>
<xml_diff>
--- a/Clipboard_v4_Master_Base.xlsx
+++ b/Clipboard_v4_Master_Base.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Clipboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\clipboard-test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FC35D3-F64A-4EDA-B5F8-29AB06F9F3E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E81E72-F931-409E-8E2F-890984BA743C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1665" yWindow="360" windowWidth="27030" windowHeight="13620" activeTab="1" xr2:uid="{366A1260-1365-4B39-9968-5A4EAE027BF5}"/>
+    <workbookView xWindow="285" yWindow="420" windowWidth="14715" windowHeight="13920" activeTab="1" xr2:uid="{B5A7B246-83E3-4800-9863-625CA16CE35B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3031" uniqueCount="977">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3044" uniqueCount="979">
   <si>
     <t>Clipboard v3.0 Master Workbook — Base Configuration</t>
   </si>
@@ -2288,9 +2288,6 @@
     <t>Pull-Down Stair</t>
   </si>
   <si>
-    <t>Mini-Split</t>
-  </si>
-  <si>
     <t>Tankless Electric</t>
   </si>
   <si>
@@ -2958,6 +2955,15 @@
   </si>
   <si>
     <t>bathroom4_updated</t>
+  </si>
+  <si>
+    <t>Vacation Rental</t>
+  </si>
+  <si>
+    <t>Inside Main Living Area</t>
+  </si>
+  <si>
+    <t>Mini-Split / Ductls</t>
   </si>
 </sst>
 </file>
@@ -3230,14 +3236,14 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4033,28 +4039,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -4162,22 +4168,23 @@
   <dimension ref="A1:R125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="12" width="9" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="38" customWidth="1"/>
-    <col min="15" max="15" width="9" customWidth="1"/>
-    <col min="16" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="22" customWidth="1"/>
-    <col min="18" max="18" width="26" customWidth="1"/>
+    <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.75" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="38.625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" x14ac:dyDescent="0.25">
@@ -4953,7 +4960,9 @@
       <c r="H16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I16" s="1"/>
+      <c r="I16" s="1" t="s">
+        <v>611</v>
+      </c>
       <c r="J16" s="1" t="s">
         <v>47</v>
       </c>
@@ -5003,7 +5012,9 @@
       <c r="H17" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I17" s="1"/>
+      <c r="I17" s="1" t="s">
+        <v>612</v>
+      </c>
       <c r="J17" s="1" t="s">
         <v>47</v>
       </c>
@@ -5203,7 +5214,9 @@
       <c r="H21" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I21" s="1"/>
+      <c r="I21" s="1" t="s">
+        <v>613</v>
+      </c>
       <c r="J21" s="1" t="s">
         <v>47</v>
       </c>
@@ -5253,7 +5266,9 @@
       <c r="H22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I22" s="1"/>
+      <c r="I22" t="s">
+        <v>613</v>
+      </c>
       <c r="J22" s="1" t="s">
         <v>47</v>
       </c>
@@ -5303,7 +5318,9 @@
       <c r="H23" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I23" s="1"/>
+      <c r="I23" t="s">
+        <v>614</v>
+      </c>
       <c r="J23" s="1" t="s">
         <v>48</v>
       </c>
@@ -5353,7 +5370,9 @@
       <c r="H24" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I24" s="1"/>
+      <c r="I24" t="s">
+        <v>615</v>
+      </c>
       <c r="J24" s="1" t="s">
         <v>48</v>
       </c>
@@ -5503,7 +5522,9 @@
       <c r="H27" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I27" s="1"/>
+      <c r="I27" s="1" t="s">
+        <v>151</v>
+      </c>
       <c r="J27" s="1" t="s">
         <v>48</v>
       </c>
@@ -5609,7 +5630,9 @@
       <c r="H29" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I29" s="1"/>
+      <c r="I29" t="s">
+        <v>617</v>
+      </c>
       <c r="J29" s="1" t="s">
         <v>47</v>
       </c>
@@ -5937,7 +5960,9 @@
       <c r="H36" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I36" s="1"/>
+      <c r="I36" t="s">
+        <v>618</v>
+      </c>
       <c r="J36" s="1" t="s">
         <v>47</v>
       </c>
@@ -5987,7 +6012,9 @@
       <c r="H37" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I37" s="1"/>
+      <c r="I37" t="s">
+        <v>619</v>
+      </c>
       <c r="J37" s="1" t="s">
         <v>48</v>
       </c>
@@ -6037,7 +6064,9 @@
       <c r="H38" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I38" s="1"/>
+      <c r="I38" t="s">
+        <v>619</v>
+      </c>
       <c r="J38" s="1" t="s">
         <v>47</v>
       </c>
@@ -6089,7 +6118,9 @@
       <c r="H39" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I39" s="1"/>
+      <c r="I39" t="s">
+        <v>620</v>
+      </c>
       <c r="J39" s="1" t="s">
         <v>48</v>
       </c>
@@ -8382,7 +8413,7 @@
       <c r="O85" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="P85" s="31" t="s">
+      <c r="P85" s="28" t="s">
         <v>48</v>
       </c>
       <c r="Q85" s="1" t="s">
@@ -9839,9 +9870,7 @@
       <c r="H115" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I115" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="I115" s="1"/>
       <c r="J115" s="1" t="s">
         <v>48</v>
       </c>
@@ -9889,9 +9918,7 @@
       <c r="H116" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I116" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="I116" s="1"/>
       <c r="J116" s="1" t="s">
         <v>48</v>
       </c>
@@ -10496,10 +10523,10 @@
         <v>40</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>966</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>967</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>968</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>46</v>
@@ -10525,10 +10552,10 @@
         <v>50</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>968</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>969</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>970</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>46</v>
@@ -10554,10 +10581,10 @@
         <v>60</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>970</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>971</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>972</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>46</v>
@@ -10583,10 +10610,10 @@
         <v>70</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>972</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>973</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>974</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>46</v>
@@ -10612,10 +10639,10 @@
         <v>80</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>975</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>976</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>46</v>
@@ -13862,7 +13889,7 @@
         <v>631</v>
       </c>
       <c r="AU2" t="s">
-        <v>638</v>
+        <v>977</v>
       </c>
       <c r="AV2" t="s">
         <v>639</v>
@@ -14074,7 +14101,7 @@
         <v>694</v>
       </c>
       <c r="AU3" t="s">
-        <v>304</v>
+        <v>638</v>
       </c>
       <c r="AV3" t="s">
         <v>695</v>
@@ -14148,7 +14175,7 @@
     </row>
     <row r="4" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>387</v>
+        <v>665</v>
       </c>
       <c r="B4" t="s">
         <v>713</v>
@@ -14286,7 +14313,7 @@
         <v>749</v>
       </c>
       <c r="AU4" t="s">
-        <v>750</v>
+        <v>304</v>
       </c>
       <c r="AV4" t="s">
         <v>751</v>
@@ -14295,28 +14322,28 @@
         <v>752</v>
       </c>
       <c r="AX4" t="s">
+        <v>978</v>
+      </c>
+      <c r="AY4" t="s">
         <v>753</v>
       </c>
-      <c r="AY4" t="s">
+      <c r="AZ4" t="s">
         <v>754</v>
       </c>
-      <c r="AZ4" t="s">
+      <c r="BA4" t="s">
         <v>755</v>
       </c>
-      <c r="BA4" t="s">
+      <c r="BB4" t="s">
         <v>756</v>
-      </c>
-      <c r="BB4" t="s">
-        <v>757</v>
       </c>
       <c r="BC4" t="s">
         <v>715</v>
       </c>
       <c r="BD4" t="s">
+        <v>757</v>
+      </c>
+      <c r="BE4" t="s">
         <v>758</v>
-      </c>
-      <c r="BE4" t="s">
-        <v>759</v>
       </c>
       <c r="BF4" t="s">
         <v>710</v>
@@ -14325,28 +14352,28 @@
         <v>710</v>
       </c>
       <c r="BH4" t="s">
+        <v>759</v>
+      </c>
+      <c r="BJ4" t="s">
         <v>760</v>
       </c>
-      <c r="BJ4" t="s">
+      <c r="BK4" t="s">
         <v>761</v>
       </c>
-      <c r="BK4" t="s">
+      <c r="BL4" t="s">
         <v>762</v>
       </c>
-      <c r="BL4" t="s">
+      <c r="BM4" t="s">
         <v>763</v>
       </c>
-      <c r="BM4" t="s">
+      <c r="BN4" t="s">
         <v>764</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BO4" t="s">
+        <v>764</v>
+      </c>
+      <c r="BP4" t="s">
         <v>765</v>
-      </c>
-      <c r="BO4" t="s">
-        <v>765</v>
-      </c>
-      <c r="BP4" t="s">
-        <v>766</v>
       </c>
       <c r="BQ4" t="s">
         <v>258</v>
@@ -14356,35 +14383,38 @@
       </c>
     </row>
     <row r="5" spans="1:70" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>387</v>
+      </c>
       <c r="B5" t="s">
+        <v>766</v>
+      </c>
+      <c r="C5" t="s">
+        <v>976</v>
+      </c>
+      <c r="D5" t="s">
         <v>767</v>
       </c>
-      <c r="C5" t="s">
-        <v>720</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>768</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>769</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>770</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>771</v>
-      </c>
-      <c r="J5" t="s">
-        <v>772</v>
       </c>
       <c r="K5" t="s">
         <v>672</v>
       </c>
       <c r="L5" t="s">
+        <v>772</v>
+      </c>
+      <c r="M5" t="s">
         <v>773</v>
-      </c>
-      <c r="M5" t="s">
-        <v>774</v>
       </c>
       <c r="N5" t="s">
         <v>631</v>
@@ -14393,145 +14423,145 @@
         <v>720</v>
       </c>
       <c r="P5" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="Q5" t="s">
         <v>720</v>
       </c>
       <c r="R5" t="s">
+        <v>775</v>
+      </c>
+      <c r="S5" t="s">
         <v>776</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>777</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>778</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>779</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>780</v>
       </c>
-      <c r="W5" t="s">
+      <c r="X5" t="s">
         <v>781</v>
       </c>
-      <c r="X5" t="s">
+      <c r="Y5" t="s">
         <v>782</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>783</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>784</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AB5" t="s">
         <v>785</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="AC5" t="s">
         <v>786</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>787</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AE5" t="s">
         <v>788</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AF5" t="s">
         <v>789</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>790</v>
       </c>
       <c r="AG5" t="s">
         <v>631</v>
       </c>
       <c r="AH5" t="s">
+        <v>790</v>
+      </c>
+      <c r="AI5" t="s">
         <v>791</v>
       </c>
-      <c r="AI5" t="s">
+      <c r="AJ5" t="s">
         <v>792</v>
       </c>
-      <c r="AJ5" t="s">
+      <c r="AK5" t="s">
         <v>793</v>
       </c>
-      <c r="AK5" t="s">
+      <c r="AL5" t="s">
         <v>794</v>
       </c>
-      <c r="AL5" t="s">
+      <c r="AM5" t="s">
         <v>795</v>
       </c>
-      <c r="AM5" t="s">
+      <c r="AN5" t="s">
         <v>796</v>
       </c>
-      <c r="AN5" t="s">
+      <c r="AO5" t="s">
         <v>797</v>
       </c>
-      <c r="AO5" t="s">
+      <c r="AP5" t="s">
         <v>798</v>
       </c>
-      <c r="AP5" t="s">
+      <c r="AQ5" t="s">
+        <v>780</v>
+      </c>
+      <c r="AR5" t="s">
         <v>799</v>
       </c>
-      <c r="AQ5" t="s">
-        <v>781</v>
-      </c>
-      <c r="AR5" t="s">
+      <c r="AS5" t="s">
         <v>800</v>
       </c>
-      <c r="AS5" t="s">
+      <c r="AT5" t="s">
         <v>801</v>
       </c>
-      <c r="AT5" t="s">
-        <v>802</v>
-      </c>
       <c r="AU5" t="s">
-        <v>626</v>
+        <v>750</v>
       </c>
       <c r="AV5" t="s">
         <v>387</v>
       </c>
       <c r="AW5" t="s">
+        <v>802</v>
+      </c>
+      <c r="AX5" t="s">
         <v>803</v>
       </c>
-      <c r="AX5" t="s">
+      <c r="AY5" t="s">
         <v>804</v>
-      </c>
-      <c r="AY5" t="s">
-        <v>805</v>
       </c>
       <c r="AZ5" t="s">
         <v>720</v>
       </c>
       <c r="BA5" t="s">
+        <v>805</v>
+      </c>
+      <c r="BB5" t="s">
         <v>806</v>
       </c>
-      <c r="BB5" t="s">
+      <c r="BC5" t="s">
         <v>807</v>
       </c>
-      <c r="BC5" t="s">
+      <c r="BD5" t="s">
         <v>808</v>
       </c>
-      <c r="BD5" t="s">
+      <c r="BE5" t="s">
         <v>809</v>
       </c>
-      <c r="BE5" t="s">
+      <c r="BF5" t="s">
         <v>810</v>
       </c>
-      <c r="BF5" t="s">
+      <c r="BG5" t="s">
+        <v>810</v>
+      </c>
+      <c r="BL5" t="s">
+        <v>964</v>
+      </c>
+      <c r="BM5" t="s">
         <v>811</v>
       </c>
-      <c r="BG5" t="s">
-        <v>811</v>
-      </c>
-      <c r="BL5" t="s">
-        <v>965</v>
-      </c>
-      <c r="BM5" t="s">
+      <c r="BN5" t="s">
         <v>812</v>
-      </c>
-      <c r="BN5" t="s">
-        <v>813</v>
       </c>
       <c r="BO5" t="s">
         <v>304</v>
@@ -14545,7 +14575,10 @@
     </row>
     <row r="6" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>814</v>
+        <v>813</v>
+      </c>
+      <c r="C6" t="s">
+        <v>720</v>
       </c>
       <c r="D6" t="s">
         <v>387</v>
@@ -14554,13 +14587,13 @@
         <v>713</v>
       </c>
       <c r="F6" t="s">
+        <v>814</v>
+      </c>
+      <c r="H6" t="s">
         <v>815</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>816</v>
-      </c>
-      <c r="J6" t="s">
-        <v>817</v>
       </c>
       <c r="K6" t="s">
         <v>726</v>
@@ -14572,76 +14605,76 @@
         <v>720</v>
       </c>
       <c r="N6" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="P6" t="s">
         <v>720</v>
       </c>
       <c r="R6" t="s">
+        <v>818</v>
+      </c>
+      <c r="S6" t="s">
         <v>819</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>820</v>
-      </c>
-      <c r="T6" t="s">
-        <v>821</v>
       </c>
       <c r="U6" t="s">
         <v>683</v>
       </c>
       <c r="V6" t="s">
+        <v>821</v>
+      </c>
+      <c r="W6" t="s">
         <v>822</v>
       </c>
-      <c r="W6" t="s">
+      <c r="X6" t="s">
         <v>823</v>
       </c>
-      <c r="X6" t="s">
+      <c r="Y6" t="s">
         <v>824</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Z6" t="s">
         <v>825</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>826</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AB6" t="s">
         <v>827</v>
       </c>
-      <c r="AB6" t="s">
+      <c r="AC6" t="s">
         <v>828</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AD6" t="s">
         <v>829</v>
       </c>
-      <c r="AD6" t="s">
+      <c r="AE6" t="s">
         <v>830</v>
       </c>
-      <c r="AE6" t="s">
+      <c r="AF6" t="s">
         <v>831</v>
       </c>
-      <c r="AF6" t="s">
+      <c r="AG6" t="s">
         <v>832</v>
       </c>
-      <c r="AG6" t="s">
+      <c r="AH6" t="s">
         <v>833</v>
       </c>
-      <c r="AH6" t="s">
-        <v>834</v>
-      </c>
       <c r="AI6" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="AJ6" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="AK6" t="s">
         <v>631</v>
       </c>
       <c r="AL6" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="AM6" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="AN6" t="s">
         <v>387</v>
@@ -14650,28 +14683,28 @@
         <v>318</v>
       </c>
       <c r="AP6" t="s">
+        <v>835</v>
+      </c>
+      <c r="AQ6" t="s">
         <v>836</v>
       </c>
-      <c r="AQ6" t="s">
+      <c r="AR6" t="s">
         <v>837</v>
       </c>
-      <c r="AR6" t="s">
+      <c r="AS6" t="s">
         <v>838</v>
-      </c>
-      <c r="AS6" t="s">
-        <v>839</v>
       </c>
       <c r="AT6" t="s">
         <v>635</v>
       </c>
       <c r="AU6" t="s">
-        <v>840</v>
+        <v>626</v>
       </c>
       <c r="AW6" t="s">
         <v>387</v>
       </c>
       <c r="AX6" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="AY6" t="s">
         <v>197</v>
@@ -14680,37 +14713,37 @@
         <v>387</v>
       </c>
       <c r="BA6" t="s">
+        <v>841</v>
+      </c>
+      <c r="BB6" t="s">
         <v>842</v>
       </c>
-      <c r="BB6" t="s">
+      <c r="BC6" t="s">
         <v>843</v>
-      </c>
-      <c r="BC6" t="s">
-        <v>844</v>
       </c>
       <c r="BD6" t="s">
         <v>387</v>
       </c>
       <c r="BE6" t="s">
+        <v>844</v>
+      </c>
+      <c r="BF6" t="s">
         <v>845</v>
       </c>
-      <c r="BF6" t="s">
-        <v>846</v>
-      </c>
       <c r="BG6" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="BL6" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="BM6" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="BN6" t="s">
         <v>626</v>
       </c>
       <c r="BO6" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="BQ6" t="s">
         <v>387</v>
@@ -14718,28 +14751,28 @@
     </row>
     <row r="7" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
+        <v>846</v>
+      </c>
+      <c r="E7" t="s">
         <v>847</v>
       </c>
-      <c r="E7" t="s">
+      <c r="H7" t="s">
+        <v>817</v>
+      </c>
+      <c r="J7" t="s">
         <v>848</v>
       </c>
-      <c r="H7" t="s">
-        <v>818</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
+        <v>775</v>
+      </c>
+      <c r="N7" t="s">
+        <v>770</v>
+      </c>
+      <c r="R7" t="s">
         <v>849</v>
       </c>
-      <c r="K7" t="s">
-        <v>776</v>
-      </c>
-      <c r="N7" t="s">
-        <v>771</v>
-      </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>850</v>
-      </c>
-      <c r="S7" t="s">
-        <v>851</v>
       </c>
       <c r="T7" t="s">
         <v>387</v>
@@ -14748,49 +14781,49 @@
         <v>627</v>
       </c>
       <c r="V7" t="s">
+        <v>851</v>
+      </c>
+      <c r="W7" t="s">
         <v>852</v>
       </c>
-      <c r="W7" t="s">
+      <c r="X7" t="s">
         <v>853</v>
-      </c>
-      <c r="X7" t="s">
-        <v>854</v>
       </c>
       <c r="Y7" t="s">
         <v>387</v>
       </c>
       <c r="Z7" t="s">
+        <v>854</v>
+      </c>
+      <c r="AA7" t="s">
         <v>855</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AB7" t="s">
         <v>856</v>
       </c>
-      <c r="AB7" t="s">
+      <c r="AC7" t="s">
         <v>857</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AD7" t="s">
         <v>858</v>
       </c>
-      <c r="AD7" t="s">
+      <c r="AE7" t="s">
         <v>859</v>
       </c>
-      <c r="AE7" t="s">
+      <c r="AF7" t="s">
         <v>860</v>
-      </c>
-      <c r="AF7" t="s">
-        <v>861</v>
       </c>
       <c r="AG7" t="s">
         <v>387</v>
       </c>
       <c r="AH7" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="AI7" t="s">
         <v>387</v>
       </c>
       <c r="AJ7" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="AK7" t="s">
         <v>627</v>
@@ -14802,25 +14835,25 @@
         <v>387</v>
       </c>
       <c r="AO7" t="s">
+        <v>863</v>
+      </c>
+      <c r="AP7" t="s">
         <v>864</v>
-      </c>
-      <c r="AP7" t="s">
-        <v>865</v>
       </c>
       <c r="AQ7" t="s">
         <v>387</v>
       </c>
       <c r="AR7" t="s">
+        <v>865</v>
+      </c>
+      <c r="AS7" t="s">
         <v>866</v>
-      </c>
-      <c r="AS7" t="s">
-        <v>867</v>
       </c>
       <c r="AT7" t="s">
         <v>387</v>
       </c>
       <c r="AU7" t="s">
-        <v>387</v>
+        <v>839</v>
       </c>
       <c r="AX7" t="s">
         <v>387</v>
@@ -14829,22 +14862,22 @@
         <v>387</v>
       </c>
       <c r="BA7" t="s">
+        <v>867</v>
+      </c>
+      <c r="BB7" t="s">
         <v>868</v>
       </c>
-      <c r="BB7" t="s">
+      <c r="BC7" t="s">
         <v>869</v>
       </c>
-      <c r="BC7" t="s">
+      <c r="BE7" t="s">
         <v>870</v>
       </c>
-      <c r="BE7" t="s">
+      <c r="BF7" t="s">
         <v>871</v>
       </c>
-      <c r="BF7" t="s">
-        <v>872</v>
-      </c>
       <c r="BG7" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="BL7" t="s">
         <v>387</v>
@@ -14853,7 +14886,7 @@
         <v>347</v>
       </c>
       <c r="BN7" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="BO7" t="s">
         <v>361</v>
@@ -14861,46 +14894,46 @@
     </row>
     <row r="8" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
+        <v>873</v>
+      </c>
+      <c r="E8" t="s">
         <v>874</v>
-      </c>
-      <c r="E8" t="s">
-        <v>875</v>
       </c>
       <c r="H8" t="s">
         <v>387</v>
       </c>
       <c r="J8" t="s">
+        <v>875</v>
+      </c>
+      <c r="K8" t="s">
+        <v>818</v>
+      </c>
+      <c r="N8" t="s">
         <v>876</v>
       </c>
-      <c r="K8" t="s">
-        <v>819</v>
-      </c>
-      <c r="N8" t="s">
+      <c r="R8" t="s">
         <v>877</v>
-      </c>
-      <c r="R8" t="s">
-        <v>878</v>
       </c>
       <c r="S8" t="s">
         <v>387</v>
       </c>
       <c r="U8" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="V8" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="W8" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="X8" t="s">
         <v>722</v>
       </c>
       <c r="Z8" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="AA8" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="AB8" t="s">
         <v>387</v>
@@ -14921,34 +14954,37 @@
         <v>749</v>
       </c>
       <c r="AJ8" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="AK8" t="s">
         <v>387</v>
       </c>
       <c r="AO8" t="s">
+        <v>881</v>
+      </c>
+      <c r="AP8" t="s">
         <v>882</v>
       </c>
-      <c r="AP8" t="s">
+      <c r="AR8" t="s">
         <v>883</v>
       </c>
-      <c r="AR8" t="s">
+      <c r="AS8" t="s">
         <v>884</v>
       </c>
-      <c r="AS8" t="s">
+      <c r="AU8" t="s">
+        <v>387</v>
+      </c>
+      <c r="BA8" t="s">
         <v>885</v>
       </c>
-      <c r="BA8" t="s">
+      <c r="BB8" t="s">
         <v>886</v>
-      </c>
-      <c r="BB8" t="s">
-        <v>887</v>
       </c>
       <c r="BC8" t="s">
         <v>387</v>
       </c>
       <c r="BE8" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="BF8" t="s">
         <v>177</v>
@@ -14957,7 +14993,7 @@
         <v>177</v>
       </c>
       <c r="BM8" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="BN8" t="s">
         <v>387</v>
@@ -14968,43 +15004,43 @@
     </row>
     <row r="9" spans="1:70" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="E9" t="s">
         <v>659</v>
       </c>
       <c r="J9" t="s">
+        <v>890</v>
+      </c>
+      <c r="K9" t="s">
         <v>891</v>
       </c>
-      <c r="K9" t="s">
+      <c r="N9" t="s">
         <v>892</v>
       </c>
-      <c r="N9" t="s">
+      <c r="R9" t="s">
         <v>893</v>
       </c>
-      <c r="R9" t="s">
-        <v>894</v>
-      </c>
       <c r="U9" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="V9" t="s">
         <v>700</v>
       </c>
       <c r="W9" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="X9" t="s">
         <v>387</v>
       </c>
       <c r="Z9" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="AA9" t="s">
         <v>387</v>
       </c>
       <c r="AH9" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="AJ9" t="s">
         <v>694</v>
@@ -15028,27 +15064,27 @@
         <v>304</v>
       </c>
       <c r="BE9" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="BF9" t="s">
         <v>387</v>
       </c>
       <c r="BG9" t="s">
+        <v>898</v>
+      </c>
+      <c r="BM9" t="s">
         <v>899</v>
-      </c>
-      <c r="BM9" t="s">
-        <v>900</v>
       </c>
     </row>
     <row r="10" spans="1:70" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="J10" t="s">
         <v>147</v>
       </c>
       <c r="K10" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="N10" t="s">
         <v>387</v>
@@ -15057,7 +15093,7 @@
         <v>387</v>
       </c>
       <c r="U10" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="V10" t="s">
         <v>387</v>
@@ -15066,7 +15102,7 @@
         <v>387</v>
       </c>
       <c r="Z10" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="AH10" t="s">
         <v>387</v>
@@ -15081,10 +15117,10 @@
         <v>387</v>
       </c>
       <c r="BB10" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="BE10" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="BG10" t="s">
         <v>387</v>
@@ -15101,10 +15137,10 @@
         <v>387</v>
       </c>
       <c r="K11" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="U11" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="Z11" t="s">
         <v>387</v>
@@ -15113,7 +15149,7 @@
         <v>387</v>
       </c>
       <c r="BB11" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="BE11" t="s">
         <v>387</v>
@@ -15124,7 +15160,7 @@
         <v>387</v>
       </c>
       <c r="U12" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="BB12" t="s">
         <v>361</v>
@@ -15132,7 +15168,7 @@
     </row>
     <row r="13" spans="1:70" x14ac:dyDescent="0.25">
       <c r="U13" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="BB13" t="s">
         <v>367</v>
@@ -15348,7 +15384,7 @@
     </row>
     <row r="1573" spans="60:60" ht="17.25" x14ac:dyDescent="0.25">
       <c r="BH1573" s="13" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="1574" spans="60:60" ht="17.25" x14ac:dyDescent="0.25">
@@ -16943,47 +16979,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>908</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>909</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>910</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>910</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>911</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>912</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>912</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>913</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>914</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>914</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>915</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>916</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>916</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>917</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>918</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>47</v>
@@ -16991,7 +17027,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>47</v>
@@ -16999,15 +17035,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>920</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>921</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>922</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>47</v>
@@ -17015,7 +17051,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>47</v>
@@ -17023,74 +17059,74 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>924</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>925</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>926</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>926</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>927</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>928</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>928</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>929</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>930</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>930</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>931</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>932</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>932</v>
+      </c>
+      <c r="B15" t="s">
         <v>933</v>
-      </c>
-      <c r="B15" t="s">
-        <v>934</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B16" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="B17" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="B18" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>937</v>
+      </c>
+      <c r="B19" t="s">
         <v>938</v>
-      </c>
-      <c r="B19" t="s">
-        <v>939</v>
       </c>
     </row>
   </sheetData>
@@ -17113,46 +17149,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>447</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>940</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>941</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>942</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -17465,7 +17501,7 @@
         <v>29</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -17473,7 +17509,7 @@
         <v>46</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -17481,7 +17517,7 @@
         <v>97</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -17489,7 +17525,7 @@
         <v>59</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -17497,7 +17533,7 @@
         <v>54</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -17505,15 +17541,15 @@
         <v>68</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>950</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>951</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>952</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -17521,7 +17557,7 @@
         <v>91</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -17529,7 +17565,7 @@
         <v>74</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -17537,15 +17573,15 @@
         <v>447</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>955</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>956</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>957</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -17553,7 +17589,7 @@
         <v>396</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -17561,15 +17597,15 @@
         <v>392</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>959</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>960</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>961</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -17577,7 +17613,7 @@
         <v>430</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
   </sheetData>
@@ -17599,7 +17635,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>25</v>
@@ -17666,7 +17702,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>